<commit_message>
updated mapper.xlsx to include columns of 'results_exp'.txt
</commit_message>
<xml_diff>
--- a/mapper.xlsx
+++ b/mapper.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anmolsoni/Documents/RegionalDSKSFC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6633D88-CA71-7849-941A-2CA27E7E5A87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C4CEB5D-3E99-D94C-B43E-8164C453FF1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="620" windowWidth="28040" windowHeight="17140" activeTab="1" xr2:uid="{7B5D8ECC-AFFD-C049-ABE8-29298D1644A4}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="2" xr2:uid="{7B5D8ECC-AFFD-C049-ABE8-29298D1644A4}"/>
   </bookViews>
   <sheets>
     <sheet name="ymc" sheetId="1" r:id="rId1"/>
     <sheet name="region_ymc" sheetId="2" r:id="rId2"/>
+    <sheet name="results_exp" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="247">
   <si>
     <t>time</t>
   </si>
@@ -412,18 +413,391 @@
   </si>
   <si>
     <t>figure_name</t>
+  </si>
+  <si>
+    <t>GDP_r</t>
+  </si>
+  <si>
+    <t>cpi_rel</t>
+  </si>
+  <si>
+    <t>Emiss_TOT</t>
+  </si>
+  <si>
+    <t>D_en_TOT</t>
+  </si>
+  <si>
+    <t>K_tot</t>
+  </si>
+  <si>
+    <t>A1p_en_dead_over_survive</t>
+  </si>
+  <si>
+    <t>A2_en_dead_over_survive</t>
+  </si>
+  <si>
+    <t>Am_en</t>
+  </si>
+  <si>
+    <t>Am_a</t>
+  </si>
+  <si>
+    <t>exit_marketshare2</t>
+  </si>
+  <si>
+    <t>exit_payments2</t>
+  </si>
+  <si>
+    <t>exit_equity2</t>
+  </si>
+  <si>
+    <t>exiting_1</t>
+  </si>
+  <si>
+    <t>baddebt_b_over_GDP</t>
+  </si>
+  <si>
+    <t>counter_bankfailure</t>
+  </si>
+  <si>
+    <t>CapitalStock_over_GDP</t>
+  </si>
+  <si>
+    <t>NW_cb_over_GDP</t>
+  </si>
+  <si>
+    <t>NW_h_over_GDP</t>
+  </si>
+  <si>
+    <t>NW_2_over_GDP</t>
+  </si>
+  <si>
+    <t>NW_b_over_GDP</t>
+  </si>
+  <si>
+    <t>BankProfits</t>
+  </si>
+  <si>
+    <t>Loans_2_over_GDP</t>
+  </si>
+  <si>
+    <t>CreditDemand_over_Supply</t>
+  </si>
+  <si>
+    <t>NW_gov_over_GDP</t>
+  </si>
+  <si>
+    <t>NW_e_over_GDP</t>
+  </si>
+  <si>
+    <t>NW_1_over_GDP</t>
+  </si>
+  <si>
+    <t>bankfailure_dummy</t>
+  </si>
+  <si>
+    <t>cpi</t>
+  </si>
+  <si>
+    <t>exp_quota</t>
+  </si>
+  <si>
+    <t>real_wage</t>
+  </si>
+  <si>
+    <t>Am2</t>
+  </si>
+  <si>
+    <t>Am1</t>
+  </si>
+  <si>
+    <t>GDP_n</t>
+  </si>
+  <si>
+    <t>Investment_n</t>
+  </si>
+  <si>
+    <t>t_CO2_en</t>
+  </si>
+  <si>
+    <t>ReplacementInvestment_r</t>
+  </si>
+  <si>
+    <t>Tmixed</t>
+  </si>
+  <si>
+    <t>EnergyPayments</t>
+  </si>
+  <si>
+    <t>FuelCost_over_GDP</t>
+  </si>
+  <si>
+    <t>GreenCapacityShare</t>
+  </si>
+  <si>
+    <t>Deposits_e_over_GDP</t>
+  </si>
+  <si>
+    <t>CapitalStock_e_over_GDP</t>
+  </si>
+  <si>
+    <t>Pitot1</t>
+  </si>
+  <si>
+    <t>Pitot2</t>
+  </si>
+  <si>
+    <t>ProfitEnergy</t>
+  </si>
+  <si>
+    <t>real_wages_total</t>
+  </si>
+  <si>
+    <t>Dividends_1</t>
+  </si>
+  <si>
+    <t>Dividends_2</t>
+  </si>
+  <si>
+    <t>Consumption_nominal</t>
+  </si>
+  <si>
+    <t>c_en</t>
+  </si>
+  <si>
+    <t>Deposits_2_over_GDP</t>
+  </si>
+  <si>
+    <t>Deposits_1_over_GDP</t>
+  </si>
+  <si>
+    <t>Deposits_firms_over_GDP</t>
+  </si>
+  <si>
+    <t>exit_total</t>
+  </si>
+  <si>
+    <t>Pitot_total</t>
+  </si>
+  <si>
+    <t>Dividends_firms_real</t>
+  </si>
+  <si>
+    <t>Dividends_energy_real</t>
+  </si>
+  <si>
+    <t>Dividends_banks_real</t>
+  </si>
+  <si>
+    <t>NW_firms_over_GDP</t>
+  </si>
+  <si>
+    <t>GovDebt_over_GDP</t>
+  </si>
+  <si>
+    <t>inflation_yoy</t>
+  </si>
+  <si>
+    <t>GDP_growth_yoy</t>
+  </si>
+  <si>
+    <t>NW_f_over_GDP</t>
+  </si>
+  <si>
+    <t>Labour_income_share</t>
+  </si>
+  <si>
+    <t>Consumption_real</t>
+  </si>
+  <si>
+    <t>Investment_real</t>
+  </si>
+  <si>
+    <t>CPI_relative</t>
+  </si>
+  <si>
+    <t>CapitalStock</t>
+  </si>
+  <si>
+    <t>ProductivityLoss_K</t>
+  </si>
+  <si>
+    <t>ProductivityLoss_C</t>
+  </si>
+  <si>
+    <t>MeanEnergyEfficiency</t>
+  </si>
+  <si>
+    <t>MeanProductivity</t>
+  </si>
+  <si>
+    <t>exit_KFirms</t>
+  </si>
+  <si>
+    <t>BailoutCost</t>
+  </si>
+  <si>
+    <t>BankFailures</t>
+  </si>
+  <si>
+    <t>CreditTightness</t>
+  </si>
+  <si>
+    <t>SystemicBankDummy</t>
+  </si>
+  <si>
+    <t>GreenExpansionQuota</t>
+  </si>
+  <si>
+    <t>RealWage</t>
+  </si>
+  <si>
+    <t>MeanProd_C</t>
+  </si>
+  <si>
+    <t>MeanProd_K</t>
+  </si>
+  <si>
+    <t>Investment_nominal</t>
+  </si>
+  <si>
+    <t>ReplacementInvestment</t>
+  </si>
+  <si>
+    <t>KFirmEmissions</t>
+  </si>
+  <si>
+    <t>CFirmEmissions</t>
+  </si>
+  <si>
+    <t>EnergyEmissions</t>
+  </si>
+  <si>
+    <t>EnergyRevenues</t>
+  </si>
+  <si>
+    <t>KFirmProfits</t>
+  </si>
+  <si>
+    <t>CFirmProfits</t>
+  </si>
+  <si>
+    <t>EnergyProfits</t>
+  </si>
+  <si>
+    <t>RealWageBill</t>
+  </si>
+  <si>
+    <t>KFirmDividends</t>
+  </si>
+  <si>
+    <t>CFirmDividends</t>
+  </si>
+  <si>
+    <t>Consumption_nominal_energy</t>
+  </si>
+  <si>
+    <t>EnergyPrice</t>
+  </si>
+  <si>
+    <t>FirmExits_total</t>
+  </si>
+  <si>
+    <t>FirmProfits_total</t>
+  </si>
+  <si>
+    <t>FirmNetWorth_GDP</t>
+  </si>
+  <si>
+    <t>Inflation_yoy</t>
+  </si>
+  <si>
+    <t>exit_marketshare_Cfirms</t>
+  </si>
+  <si>
+    <t>exit_payment_Cfirms</t>
+  </si>
+  <si>
+    <t>exit_equity_Cfirms</t>
+  </si>
+  <si>
+    <t>CfirmLoans/GDP</t>
+  </si>
+  <si>
+    <t>Bank_NetWorth/GDP</t>
+  </si>
+  <si>
+    <t>CFirm_NetWorth/GDP</t>
+  </si>
+  <si>
+    <t>Household_NetWorth/GDP</t>
+  </si>
+  <si>
+    <t>CB_NetWorth/GDP</t>
+  </si>
+  <si>
+    <t>Capital/GDP</t>
+  </si>
+  <si>
+    <t>BankBadDebt/GDP</t>
+  </si>
+  <si>
+    <t>Government_NetWorth/GDP</t>
+  </si>
+  <si>
+    <t>Energy_NetWorth/GDP</t>
+  </si>
+  <si>
+    <t>KFirm_NetWorth/GDP</t>
+  </si>
+  <si>
+    <t>CarbonTaxon EnergySector</t>
+  </si>
+  <si>
+    <t>FuelCost/GDP</t>
+  </si>
+  <si>
+    <t>EnergyDeposits/GDP</t>
+  </si>
+  <si>
+    <t>EnergyCapital/GDP</t>
+  </si>
+  <si>
+    <t>CFirmDeposits/GDP</t>
+  </si>
+  <si>
+    <t>KFirmDeposits/GDP</t>
+  </si>
+  <si>
+    <t>FirmDeposits/GDP</t>
+  </si>
+  <si>
+    <t>GovDebt/GDP</t>
+  </si>
+  <si>
+    <t>FossilFuel_NetWorth/GDP</t>
+  </si>
+  <si>
+    <t>LabourIncomeShare</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -447,8 +821,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1515,4 +1890,618 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB204543-0B37-7F48-A08B-75000A6D4A29}">
+  <dimension ref="A1:B75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>126</v>
+      </c>
+      <c r="B7" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>127</v>
+      </c>
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>129</v>
+      </c>
+      <c r="B11" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>130</v>
+      </c>
+      <c r="B12" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>131</v>
+      </c>
+      <c r="B13" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B14" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>133</v>
+      </c>
+      <c r="B15" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>134</v>
+      </c>
+      <c r="B16" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>135</v>
+      </c>
+      <c r="B17" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>136</v>
+      </c>
+      <c r="B18" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>137</v>
+      </c>
+      <c r="B19" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>138</v>
+      </c>
+      <c r="B21" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>139</v>
+      </c>
+      <c r="B22" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>140</v>
+      </c>
+      <c r="B23" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>141</v>
+      </c>
+      <c r="B24" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>142</v>
+      </c>
+      <c r="B25" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>143</v>
+      </c>
+      <c r="B26" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>144</v>
+      </c>
+      <c r="B27" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>145</v>
+      </c>
+      <c r="B28" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>146</v>
+      </c>
+      <c r="B29" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>147</v>
+      </c>
+      <c r="B30" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>148</v>
+      </c>
+      <c r="B31" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>149</v>
+      </c>
+      <c r="B32" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>150</v>
+      </c>
+      <c r="B33" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>151</v>
+      </c>
+      <c r="B34" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>152</v>
+      </c>
+      <c r="B35" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>153</v>
+      </c>
+      <c r="B36" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>154</v>
+      </c>
+      <c r="B37" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>155</v>
+      </c>
+      <c r="B38" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>156</v>
+      </c>
+      <c r="B39" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>157</v>
+      </c>
+      <c r="B40" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>158</v>
+      </c>
+      <c r="B41" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>2</v>
+      </c>
+      <c r="B42" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>159</v>
+      </c>
+      <c r="B43" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>160</v>
+      </c>
+      <c r="B44" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>96</v>
+      </c>
+      <c r="B45" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>97</v>
+      </c>
+      <c r="B46" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>98</v>
+      </c>
+      <c r="B47" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>161</v>
+      </c>
+      <c r="B48" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>162</v>
+      </c>
+      <c r="B49" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>163</v>
+      </c>
+      <c r="B50" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>164</v>
+      </c>
+      <c r="B51" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>165</v>
+      </c>
+      <c r="B52" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>166</v>
+      </c>
+      <c r="B53" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>167</v>
+      </c>
+      <c r="B54" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>168</v>
+      </c>
+      <c r="B55" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>169</v>
+      </c>
+      <c r="B56" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>170</v>
+      </c>
+      <c r="B57" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>171</v>
+      </c>
+      <c r="B58" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>172</v>
+      </c>
+      <c r="B59" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>173</v>
+      </c>
+      <c r="B60" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>174</v>
+      </c>
+      <c r="B61" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>175</v>
+      </c>
+      <c r="B62" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>176</v>
+      </c>
+      <c r="B63" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>177</v>
+      </c>
+      <c r="B64" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>178</v>
+      </c>
+      <c r="B65" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>179</v>
+      </c>
+      <c r="B66" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>180</v>
+      </c>
+      <c r="B67" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>181</v>
+      </c>
+      <c r="B68" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>182</v>
+      </c>
+      <c r="B69" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>183</v>
+      </c>
+      <c r="B70" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>184</v>
+      </c>
+      <c r="B71" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>185</v>
+      </c>
+      <c r="B72" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>186</v>
+      </c>
+      <c r="B73" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>187</v>
+      </c>
+      <c r="B74" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>188</v>
+      </c>
+      <c r="B75" t="s">
+        <v>246</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add input JSON files for heterogeneous regions scenarios
- Created scenario1_inputs.json for large more exposed regions with detailed parameters, climate parameters, shock parameters, flags, initial conditions, and climate initial conditions.
- Created scenario1_inputs.json for small more exposed regions with similar structure and parameters as the large regions file.
</commit_message>
<xml_diff>
--- a/mapper.xlsx
+++ b/mapper.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anmolsoni/Documents/RegionalDSKSFC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C943B69-F8E2-7D46-BABB-78176D0A17D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F1ED43F-237E-4C4C-9ABB-EDD40D2C84DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="4" xr2:uid="{7B5D8ECC-AFFD-C049-ABE8-29298D1644A4}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="1" xr2:uid="{7B5D8ECC-AFFD-C049-ABE8-29298D1644A4}"/>
   </bookViews>
   <sheets>
     <sheet name="ymc" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="207">
   <si>
     <t>time</t>
   </si>
@@ -171,54 +171,18 @@
     <t>reg_EmploymentRate</t>
   </si>
   <si>
-    <t>reg_Am</t>
-  </si>
-  <si>
-    <t>reg_Loans_2</t>
-  </si>
-  <si>
-    <t>reg_Inventories</t>
-  </si>
-  <si>
-    <t>reg_N</t>
-  </si>
-  <si>
     <t>reg_GDP_n</t>
   </si>
   <si>
-    <t>reg_Q_ge_over_D_en</t>
-  </si>
-  <si>
     <t>reg_D_en_TOT</t>
   </si>
   <si>
     <t>reg_Emiss_TOT</t>
   </si>
   <si>
-    <t>reg_Cum_emissions</t>
-  </si>
-  <si>
-    <t>reg_Q1</t>
-  </si>
-  <si>
-    <t>reg_Q2</t>
-  </si>
-  <si>
-    <t>reg_N1</t>
-  </si>
-  <si>
-    <t>reg_N2</t>
-  </si>
-  <si>
     <t>reg_LS</t>
   </si>
   <si>
-    <t>reg_Q_ge</t>
-  </si>
-  <si>
-    <t>reg_Q_de</t>
-  </si>
-  <si>
     <t>reg_Emiss1_TOT</t>
   </si>
   <si>
@@ -228,27 +192,12 @@
     <t>reg_Emiss_en</t>
   </si>
   <si>
-    <t>GDP_r_1</t>
-  </si>
-  <si>
     <t>Consumption_r</t>
   </si>
   <si>
     <t>Investment_r</t>
   </si>
   <si>
-    <t>EmploymentRate_1</t>
-  </si>
-  <si>
-    <t>cpi_1</t>
-  </si>
-  <si>
-    <t>cpi_1_over_cpi_2</t>
-  </si>
-  <si>
-    <t>Am_1</t>
-  </si>
-  <si>
     <t>Deficit</t>
   </si>
   <si>
@@ -258,57 +207,24 @@
     <t>w_1</t>
   </si>
   <si>
-    <t>w_1_over_w_2</t>
-  </si>
-  <si>
     <t>r</t>
   </si>
   <si>
     <t>r_bonds</t>
   </si>
   <si>
-    <t>Loans_2_Row1_Sum</t>
-  </si>
-  <si>
-    <t>Deposits_Row1_Sum</t>
-  </si>
-  <si>
-    <t>baddebt_b_Sum</t>
-  </si>
-  <si>
     <t>CreditSupply_all</t>
   </si>
   <si>
     <t>CreditDemand_all</t>
   </si>
   <si>
-    <t>Inventories_Row1_Sum</t>
-  </si>
-  <si>
-    <t>N_Row1_Sum</t>
-  </si>
-  <si>
     <t>Bailout</t>
   </si>
   <si>
-    <t>GDP_n_1</t>
-  </si>
-  <si>
-    <t>Q_ge_over_D_en_TOT_1</t>
-  </si>
-  <si>
-    <t>D_en_TOT_1</t>
-  </si>
-  <si>
-    <t>Emiss_TOT_1</t>
-  </si>
-  <si>
     <t>Cum_emissions</t>
   </si>
   <si>
-    <t>Tmixed_1</t>
-  </si>
-  <si>
     <t>Q1tot</t>
   </si>
   <si>
@@ -721,13 +637,37 @@
   </si>
   <si>
     <t>results_exp_reg</t>
+  </si>
+  <si>
+    <t>real_wage_rate</t>
+  </si>
+  <si>
+    <t>Deposits1</t>
+  </si>
+  <si>
+    <t>baddebt_b</t>
+  </si>
+  <si>
+    <t>Inventories_real</t>
+  </si>
+  <si>
+    <t>Am</t>
+  </si>
+  <si>
+    <t>Loans2</t>
+  </si>
+  <si>
+    <t>Loans_2</t>
+  </si>
+  <si>
+    <t>Inventories_r</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -748,6 +688,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0000FF"/>
+      <name val="Menlo"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -770,10 +716,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1118,13 +1065,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>122</v>
+        <v>94</v>
       </c>
       <c r="B1" t="s">
-        <v>123</v>
+        <v>95</v>
       </c>
       <c r="C1" t="s">
-        <v>124</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -1143,7 +1090,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
@@ -1154,7 +1101,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="C4" t="s">
         <v>2</v>
@@ -1165,7 +1112,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
         <v>3</v>
@@ -1176,7 +1123,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="C6" t="s">
         <v>4</v>
@@ -1187,7 +1134,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>66</v>
+        <v>112</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
@@ -1198,7 +1145,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>67</v>
+        <v>98</v>
       </c>
       <c r="C8" t="s">
         <v>6</v>
@@ -1209,7 +1156,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>68</v>
+        <v>203</v>
       </c>
       <c r="C9" t="s">
         <v>7</v>
@@ -1220,7 +1167,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>69</v>
+        <v>52</v>
       </c>
       <c r="C10" t="s">
         <v>8</v>
@@ -1231,7 +1178,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="C11" t="s">
         <v>9</v>
@@ -1242,7 +1189,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="C12" t="s">
         <v>10</v>
@@ -1252,8 +1199,8 @@
       <c r="A13">
         <v>11</v>
       </c>
-      <c r="B13" t="s">
-        <v>72</v>
+      <c r="B13" s="3" t="s">
+        <v>199</v>
       </c>
       <c r="C13" t="s">
         <v>11</v>
@@ -1264,7 +1211,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="C14" t="s">
         <v>12</v>
@@ -1275,7 +1222,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="C15" t="s">
         <v>13</v>
@@ -1286,7 +1233,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>75</v>
+        <v>204</v>
       </c>
       <c r="C16" t="s">
         <v>14</v>
@@ -1297,7 +1244,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>76</v>
+        <v>200</v>
       </c>
       <c r="C17" t="s">
         <v>15</v>
@@ -1308,7 +1255,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>77</v>
+        <v>201</v>
       </c>
       <c r="C18" t="s">
         <v>16</v>
@@ -1319,7 +1266,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="C19" t="s">
         <v>17</v>
@@ -1330,7 +1277,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>79</v>
+        <v>58</v>
       </c>
       <c r="C20" t="s">
         <v>18</v>
@@ -1341,7 +1288,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>80</v>
+        <v>19</v>
       </c>
       <c r="C21" t="s">
         <v>19</v>
@@ -1352,7 +1299,7 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>81</v>
+        <v>202</v>
       </c>
       <c r="C22" t="s">
         <v>20</v>
@@ -1363,7 +1310,7 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="C23" t="s">
         <v>21</v>
@@ -1374,7 +1321,7 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="C24" t="s">
         <v>22</v>
@@ -1385,7 +1332,7 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>84</v>
+        <v>122</v>
       </c>
       <c r="C25" t="s">
         <v>23</v>
@@ -1396,7 +1343,7 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="C26" t="s">
         <v>24</v>
@@ -1407,7 +1354,7 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="C27" t="s">
         <v>25</v>
@@ -1418,7 +1365,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>87</v>
+        <v>60</v>
       </c>
       <c r="C28" t="s">
         <v>26</v>
@@ -1429,7 +1376,7 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>88</v>
+        <v>120</v>
       </c>
       <c r="C29" t="s">
         <v>27</v>
@@ -1440,7 +1387,7 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="C30" t="s">
         <v>28</v>
@@ -1451,7 +1398,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="C31" t="s">
         <v>29</v>
@@ -1462,7 +1409,7 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="C32" t="s">
         <v>30</v>
@@ -1473,7 +1420,7 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>92</v>
+        <v>64</v>
       </c>
       <c r="C33" t="s">
         <v>31</v>
@@ -1484,7 +1431,7 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>93</v>
+        <v>65</v>
       </c>
       <c r="C34" t="s">
         <v>32</v>
@@ -1495,7 +1442,7 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>94</v>
+        <v>66</v>
       </c>
       <c r="C35" t="s">
         <v>33</v>
@@ -1506,7 +1453,7 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>95</v>
+        <v>67</v>
       </c>
       <c r="C36" t="s">
         <v>34</v>
@@ -1517,7 +1464,7 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="C37" t="s">
         <v>35</v>
@@ -1528,7 +1475,7 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="C38" t="s">
         <v>36</v>
@@ -1539,7 +1486,7 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>98</v>
+        <v>70</v>
       </c>
       <c r="C39" t="s">
         <v>37</v>
@@ -1563,13 +1510,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>122</v>
+        <v>94</v>
       </c>
       <c r="B1" t="s">
-        <v>123</v>
+        <v>95</v>
       </c>
       <c r="C1" t="s">
-        <v>124</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -1588,10 +1535,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
-        <v>99</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -1599,10 +1546,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>100</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -1610,10 +1557,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -1624,7 +1571,7 @@
         <v>42</v>
       </c>
       <c r="C6" t="s">
-        <v>102</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -1632,10 +1579,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>203</v>
       </c>
       <c r="C7" t="s">
-        <v>103</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -1643,10 +1590,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>44</v>
+        <v>205</v>
       </c>
       <c r="C8" t="s">
-        <v>104</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -1654,10 +1601,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -1665,10 +1612,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>46</v>
+        <v>206</v>
       </c>
       <c r="C10" t="s">
-        <v>106</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -1676,21 +1623,21 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>107</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>10</v>
       </c>
-      <c r="B12" t="s">
-        <v>48</v>
+      <c r="B12" s="3" t="s">
+        <v>122</v>
       </c>
       <c r="C12" t="s">
-        <v>108</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -1698,10 +1645,10 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>100</v>
       </c>
       <c r="C13" t="s">
-        <v>109</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -1709,10 +1656,10 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>50</v>
+        <v>99</v>
       </c>
       <c r="C14" t="s">
-        <v>110</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -1720,32 +1667,32 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C15" t="s">
-        <v>111</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>14</v>
       </c>
-      <c r="B16" t="s">
-        <v>52</v>
+      <c r="B16" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="C16" t="s">
-        <v>112</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>15</v>
       </c>
-      <c r="B17" t="s">
-        <v>53</v>
+      <c r="B17" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="C17" t="s">
-        <v>113</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -1753,10 +1700,10 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="C18" t="s">
-        <v>114</v>
+        <v>86</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -1764,10 +1711,10 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="C19" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -1775,10 +1722,10 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="C20" t="s">
-        <v>116</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
@@ -1786,10 +1733,10 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="C21" t="s">
-        <v>117</v>
+        <v>89</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
@@ -1797,10 +1744,10 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="C22" t="s">
-        <v>118</v>
+        <v>90</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
@@ -1808,10 +1755,10 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C23" t="s">
-        <v>119</v>
+        <v>91</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -1819,10 +1766,10 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="C24" t="s">
-        <v>120</v>
+        <v>92</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
@@ -1830,10 +1777,10 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C25" t="s">
-        <v>121</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1853,7 +1800,7 @@
   <sheetData>
     <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>123</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
@@ -1863,17 +1810,17 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>125</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
@@ -1883,177 +1830,177 @@
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>126</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>128</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>129</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>186</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>187</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>130</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>131</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>132</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>133</v>
+        <v>105</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>134</v>
+        <v>106</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>135</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>82</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>197</v>
+        <v>169</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>136</v>
+        <v>108</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>198</v>
+        <v>170</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>199</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>191</v>
+        <v>163</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>189</v>
+        <v>161</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>190</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>200</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>201</v>
+        <v>173</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>202</v>
+        <v>174</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>203</v>
+        <v>175</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>204</v>
+        <v>176</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>139</v>
+        <v>111</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>140</v>
+        <v>112</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>141</v>
+        <v>113</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>142</v>
+        <v>114</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>143</v>
+        <v>115</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>144</v>
+        <v>116</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>145</v>
+        <v>117</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>215</v>
+        <v>187</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.2">
@@ -2063,168 +2010,168 @@
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>146</v>
+        <v>118</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>147</v>
+        <v>119</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>97</v>
+        <v>69</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>98</v>
+        <v>70</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>148</v>
+        <v>120</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>149</v>
+        <v>121</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>162</v>
+        <v>134</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>150</v>
+        <v>122</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>205</v>
+        <v>177</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>206</v>
+        <v>178</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>151</v>
+        <v>123</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>152</v>
+        <v>124</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>153</v>
+        <v>125</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>217</v>
+        <v>189</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>154</v>
+        <v>126</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>155</v>
+        <v>127</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>156</v>
+        <v>128</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>157</v>
+        <v>129</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>207</v>
+        <v>179</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>208</v>
+        <v>180</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>209</v>
+        <v>181</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>158</v>
+        <v>130</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>159</v>
+        <v>131</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>160</v>
+        <v>132</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>221</v>
+        <v>193</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>222</v>
+        <v>194</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>210</v>
+        <v>182</v>
       </c>
       <c r="C70" s="2"/>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>163</v>
+        <v>135</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>211</v>
+        <v>183</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>218</v>
+        <v>190</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>212</v>
+        <v>184</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>161</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -2244,7 +2191,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>123</v>
+        <v>95</v>
       </c>
       <c r="B1" s="1"/>
     </row>
@@ -2275,207 +2222,207 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>164</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>185</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>188</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>165</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>166</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>167</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>168</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>169</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>170</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>192</v>
+        <v>164</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>193</v>
+        <v>165</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>194</v>
+        <v>166</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>195</v>
+        <v>167</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>213</v>
+        <v>185</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>196</v>
+        <v>168</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>171</v>
+        <v>143</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>172</v>
+        <v>144</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>214</v>
+        <v>186</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>216</v>
+        <v>188</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>173</v>
+        <v>145</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>174</v>
+        <v>146</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>175</v>
+        <v>147</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>176</v>
+        <v>148</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>177</v>
+        <v>149</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>178</v>
+        <v>150</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>179</v>
+        <v>151</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>180</v>
+        <v>152</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>181</v>
+        <v>153</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>182</v>
+        <v>154</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>183</v>
+        <v>155</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>223</v>
+        <v>195</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>224</v>
+        <v>196</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>220</v>
+        <v>192</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>219</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -2496,10 +2443,10 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>226</v>
+        <v>198</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>225</v>
+        <v>197</v>
       </c>
       <c r="D1" s="1"/>
     </row>
@@ -2516,7 +2463,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>125</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -2524,7 +2471,7 @@
         <v>40</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -2532,7 +2479,7 @@
         <v>41</v>
       </c>
       <c r="B5" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -2545,183 +2492,183 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
-        <v>128</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>93</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>164</v>
+        <v>136</v>
       </c>
       <c r="B10" t="s">
-        <v>129</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>185</v>
+        <v>157</v>
       </c>
       <c r="B11" t="s">
-        <v>184</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>188</v>
+        <v>160</v>
       </c>
       <c r="B12" t="s">
-        <v>187</v>
+        <v>159</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>165</v>
+        <v>137</v>
       </c>
       <c r="B13" t="s">
-        <v>130</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>166</v>
+        <v>138</v>
       </c>
       <c r="B14" t="s">
-        <v>131</v>
+        <v>103</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>167</v>
+        <v>139</v>
       </c>
       <c r="B15" t="s">
-        <v>132</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>168</v>
+        <v>140</v>
       </c>
       <c r="B16" t="s">
-        <v>133</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>169</v>
+        <v>141</v>
       </c>
       <c r="B17" t="s">
-        <v>134</v>
+        <v>106</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>170</v>
+        <v>142</v>
       </c>
       <c r="B18" t="s">
-        <v>135</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>192</v>
+        <v>164</v>
       </c>
       <c r="B19" t="s">
-        <v>137</v>
+        <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>193</v>
+        <v>165</v>
       </c>
       <c r="B20" t="s">
-        <v>191</v>
+        <v>163</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>194</v>
+        <v>166</v>
       </c>
       <c r="B21" t="s">
-        <v>189</v>
+        <v>161</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>195</v>
+        <v>167</v>
       </c>
       <c r="B22" t="s">
-        <v>200</v>
+        <v>172</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>213</v>
+        <v>185</v>
       </c>
       <c r="B23" t="s">
-        <v>201</v>
+        <v>173</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>196</v>
+        <v>168</v>
       </c>
       <c r="B24" t="s">
-        <v>204</v>
+        <v>176</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>171</v>
+        <v>143</v>
       </c>
       <c r="B25" t="s">
-        <v>143</v>
+        <v>115</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>172</v>
+        <v>144</v>
       </c>
       <c r="B26" t="s">
-        <v>144</v>
+        <v>116</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B27" t="s">
-        <v>145</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>214</v>
+        <v>186</v>
       </c>
       <c r="B28" t="s">
-        <v>215</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>216</v>
+        <v>188</v>
       </c>
       <c r="B29" t="s">
         <v>2</v>
@@ -2729,146 +2676,146 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>173</v>
+        <v>145</v>
       </c>
       <c r="B30" t="s">
-        <v>147</v>
+        <v>119</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="B31" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="B32" t="s">
-        <v>97</v>
+        <v>69</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="B33" t="s">
-        <v>98</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>174</v>
+        <v>146</v>
       </c>
       <c r="B34" t="s">
-        <v>149</v>
+        <v>121</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>175</v>
+        <v>147</v>
       </c>
       <c r="B35" t="s">
-        <v>150</v>
+        <v>122</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>176</v>
+        <v>148</v>
       </c>
       <c r="B36" t="s">
-        <v>151</v>
+        <v>123</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>177</v>
+        <v>149</v>
       </c>
       <c r="B37" t="s">
-        <v>152</v>
+        <v>124</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>178</v>
+        <v>150</v>
       </c>
       <c r="B38" t="s">
-        <v>217</v>
+        <v>189</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>179</v>
+        <v>151</v>
       </c>
       <c r="B39" t="s">
-        <v>154</v>
+        <v>126</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>180</v>
+        <v>152</v>
       </c>
       <c r="B40" t="s">
-        <v>155</v>
+        <v>127</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>181</v>
+        <v>153</v>
       </c>
       <c r="B41" t="s">
-        <v>158</v>
+        <v>130</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>182</v>
+        <v>154</v>
       </c>
       <c r="B42" t="s">
-        <v>159</v>
+        <v>131</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>183</v>
+        <v>155</v>
       </c>
       <c r="B43" t="s">
-        <v>160</v>
+        <v>132</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>223</v>
+        <v>195</v>
       </c>
       <c r="B44" t="s">
-        <v>221</v>
+        <v>193</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>224</v>
+        <v>196</v>
       </c>
       <c r="B45" t="s">
-        <v>222</v>
+        <v>194</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>220</v>
+        <v>192</v>
       </c>
       <c r="B46" t="s">
-        <v>210</v>
+        <v>182</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>219</v>
+        <v>191</v>
       </c>
       <c r="B47" t="s">
-        <v>218</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>